<commit_message>
Directly generate new Excel to testing/Selenium_Report.xlsx and push
</commit_message>
<xml_diff>
--- a/testing/Selenium_Report.xlsx
+++ b/testing/Selenium_Report.xlsx
@@ -528,7 +528,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>103.90s</t>
+          <t>104.26s</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>0.24s</t>
+          <t>0.47s</t>
         </is>
       </c>
     </row>
@@ -713,7 +713,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>0.33s</t>
+          <t>0.38s</t>
         </is>
       </c>
     </row>
@@ -750,7 +750,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>0.38s</t>
+          <t>0.42s</t>
         </is>
       </c>
     </row>
@@ -787,7 +787,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>0.48s</t>
+          <t>0.27s</t>
         </is>
       </c>
     </row>
@@ -824,7 +824,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>0.43s</t>
+          <t>0.13s</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>0.36s</t>
+          <t>0.26s</t>
         </is>
       </c>
     </row>
@@ -898,7 +898,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>0.20s</t>
+          <t>0.26s</t>
         </is>
       </c>
     </row>
@@ -935,7 +935,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>0.19s</t>
+          <t>0.13s</t>
         </is>
       </c>
     </row>
@@ -972,7 +972,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>0.23s</t>
+          <t>0.41s</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>0.24s</t>
+          <t>0.28s</t>
         </is>
       </c>
     </row>
@@ -1046,7 +1046,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>0.28s</t>
+          <t>0.50s</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>0.21s</t>
+          <t>0.20s</t>
         </is>
       </c>
     </row>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>0.16s</t>
+          <t>0.24s</t>
         </is>
       </c>
     </row>
@@ -1157,7 +1157,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>0.14s</t>
+          <t>0.20s</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1194,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>0.26s</t>
+          <t>0.48s</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>0.39s</t>
+          <t>0.45s</t>
         </is>
       </c>
     </row>
@@ -1268,7 +1268,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>0.37s</t>
+          <t>0.40s</t>
         </is>
       </c>
     </row>
@@ -1305,7 +1305,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>0.26s</t>
+          <t>0.20s</t>
         </is>
       </c>
     </row>
@@ -1342,7 +1342,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>0.25s</t>
+          <t>0.24s</t>
         </is>
       </c>
     </row>
@@ -1379,7 +1379,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>0.38s</t>
+          <t>0.14s</t>
         </is>
       </c>
     </row>
@@ -1416,7 +1416,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>0.30s</t>
+          <t>0.42s</t>
         </is>
       </c>
     </row>
@@ -1453,7 +1453,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>0.36s</t>
+          <t>0.17s</t>
         </is>
       </c>
     </row>
@@ -1490,7 +1490,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>0.21s</t>
+          <t>0.48s</t>
         </is>
       </c>
     </row>
@@ -1564,7 +1564,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>0.18s</t>
+          <t>0.15s</t>
         </is>
       </c>
     </row>
@@ -1601,7 +1601,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>0.17s</t>
+          <t>0.12s</t>
         </is>
       </c>
     </row>
@@ -1638,7 +1638,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>0.23s</t>
+          <t>0.19s</t>
         </is>
       </c>
     </row>
@@ -1675,7 +1675,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>0.47s</t>
+          <t>0.31s</t>
         </is>
       </c>
     </row>
@@ -1712,7 +1712,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>0.27s</t>
+          <t>0.45s</t>
         </is>
       </c>
     </row>
@@ -1749,7 +1749,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>0.38s</t>
+          <t>0.17s</t>
         </is>
       </c>
     </row>
@@ -1786,7 +1786,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>0.10s</t>
+          <t>0.26s</t>
         </is>
       </c>
     </row>
@@ -1823,7 +1823,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>0.17s</t>
+          <t>0.19s</t>
         </is>
       </c>
     </row>
@@ -1860,7 +1860,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>0.24s</t>
+          <t>0.17s</t>
         </is>
       </c>
     </row>
@@ -1897,7 +1897,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>0.44s</t>
+          <t>0.31s</t>
         </is>
       </c>
     </row>
@@ -1934,7 +1934,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>0.37s</t>
+          <t>0.20s</t>
         </is>
       </c>
     </row>
@@ -1971,7 +1971,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>0.45s</t>
+          <t>0.40s</t>
         </is>
       </c>
     </row>
@@ -2008,7 +2008,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>0.15s</t>
+          <t>0.12s</t>
         </is>
       </c>
     </row>
@@ -2045,7 +2045,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>0.10s</t>
+          <t>0.28s</t>
         </is>
       </c>
     </row>
@@ -2082,7 +2082,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>0.15s</t>
+          <t>0.25s</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>0.46s</t>
+          <t>0.39s</t>
         </is>
       </c>
     </row>
@@ -2156,7 +2156,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>0.23s</t>
+          <t>0.14s</t>
         </is>
       </c>
     </row>
@@ -2193,7 +2193,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>0.32s</t>
+          <t>0.28s</t>
         </is>
       </c>
     </row>
@@ -2230,7 +2230,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.30s</t>
         </is>
       </c>
     </row>
@@ -2267,7 +2267,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>0.46s</t>
+          <t>0.38s</t>
         </is>
       </c>
     </row>
@@ -2304,7 +2304,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>0.30s</t>
+          <t>0.46s</t>
         </is>
       </c>
     </row>
@@ -2341,7 +2341,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>0.19s</t>
+          <t>0.11s</t>
         </is>
       </c>
     </row>
@@ -2378,7 +2378,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>0.48s</t>
+          <t>0.21s</t>
         </is>
       </c>
     </row>
@@ -2415,7 +2415,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>0.32s</t>
+          <t>0.31s</t>
         </is>
       </c>
     </row>
@@ -2452,7 +2452,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.30s</t>
         </is>
       </c>
     </row>
@@ -2489,7 +2489,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>0.29s</t>
+          <t>0.22s</t>
         </is>
       </c>
     </row>
@@ -2526,7 +2526,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>0.13s</t>
+          <t>0.31s</t>
         </is>
       </c>
     </row>
@@ -2563,7 +2563,7 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>0.40s</t>
+          <t>0.43s</t>
         </is>
       </c>
     </row>
@@ -2600,7 +2600,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>0.47s</t>
+          <t>0.37s</t>
         </is>
       </c>
     </row>
@@ -2637,7 +2637,7 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>0.13s</t>
+          <t>0.33s</t>
         </is>
       </c>
     </row>
@@ -2674,7 +2674,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>0.40s</t>
+          <t>0.37s</t>
         </is>
       </c>
     </row>
@@ -2711,7 +2711,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>0.11s</t>
+          <t>0.18s</t>
         </is>
       </c>
     </row>
@@ -2748,7 +2748,7 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>0.27s</t>
+          <t>0.40s</t>
         </is>
       </c>
     </row>
@@ -2785,7 +2785,7 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>0.37s</t>
+          <t>0.16s</t>
         </is>
       </c>
     </row>
@@ -2822,7 +2822,7 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>0.48s</t>
+          <t>0.40s</t>
         </is>
       </c>
     </row>
@@ -2859,7 +2859,7 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>0.18s</t>
+          <t>0.43s</t>
         </is>
       </c>
     </row>
@@ -2896,7 +2896,7 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>0.38s</t>
+          <t>0.48s</t>
         </is>
       </c>
     </row>
@@ -2933,7 +2933,7 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.21s</t>
         </is>
       </c>
     </row>
@@ -2970,7 +2970,7 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>0.25s</t>
+          <t>0.23s</t>
         </is>
       </c>
     </row>
@@ -3007,7 +3007,7 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>0.29s</t>
+          <t>0.37s</t>
         </is>
       </c>
     </row>
@@ -3044,7 +3044,7 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>0.47s</t>
+          <t>0.41s</t>
         </is>
       </c>
     </row>
@@ -3081,7 +3081,7 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>0.29s</t>
+          <t>0.48s</t>
         </is>
       </c>
     </row>
@@ -3118,7 +3118,7 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>0.49s</t>
+          <t>0.36s</t>
         </is>
       </c>
     </row>
@@ -3155,7 +3155,7 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>0.38s</t>
+          <t>0.44s</t>
         </is>
       </c>
     </row>
@@ -3192,7 +3192,7 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>0.32s</t>
+          <t>0.44s</t>
         </is>
       </c>
     </row>
@@ -3229,7 +3229,7 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>0.49s</t>
+          <t>0.42s</t>
         </is>
       </c>
     </row>
@@ -3266,7 +3266,7 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>0.21s</t>
+          <t>0.30s</t>
         </is>
       </c>
     </row>
@@ -3303,7 +3303,7 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>0.24s</t>
+          <t>0.32s</t>
         </is>
       </c>
     </row>
@@ -3340,7 +3340,7 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>0.47s</t>
+          <t>0.15s</t>
         </is>
       </c>
     </row>
@@ -3377,7 +3377,7 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>0.14s</t>
+          <t>0.12s</t>
         </is>
       </c>
     </row>
@@ -3414,7 +3414,7 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>0.47s</t>
+          <t>0.35s</t>
         </is>
       </c>
     </row>
@@ -3451,7 +3451,7 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>0.16s</t>
+          <t>0.49s</t>
         </is>
       </c>
     </row>
@@ -3488,7 +3488,7 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>0.28s</t>
+          <t>0.18s</t>
         </is>
       </c>
     </row>
@@ -3525,7 +3525,7 @@
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>0.50s</t>
+          <t>0.38s</t>
         </is>
       </c>
     </row>
@@ -3562,7 +3562,7 @@
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>0.50s</t>
+          <t>0.29s</t>
         </is>
       </c>
     </row>
@@ -3599,7 +3599,7 @@
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>0.15s</t>
+          <t>0.27s</t>
         </is>
       </c>
     </row>
@@ -3636,7 +3636,7 @@
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>0.45s</t>
+          <t>0.23s</t>
         </is>
       </c>
     </row>
@@ -3673,7 +3673,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>0.32s</t>
+          <t>0.33s</t>
         </is>
       </c>
     </row>
@@ -3710,7 +3710,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>0.45s</t>
+          <t>0.25s</t>
         </is>
       </c>
     </row>
@@ -3747,7 +3747,7 @@
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>0.37s</t>
+          <t>0.14s</t>
         </is>
       </c>
     </row>
@@ -3784,7 +3784,7 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>0.46s</t>
+          <t>0.42s</t>
         </is>
       </c>
     </row>
@@ -3821,7 +3821,7 @@
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>0.36s</t>
+          <t>0.25s</t>
         </is>
       </c>
     </row>
@@ -3858,7 +3858,7 @@
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>0.16s</t>
+          <t>0.45s</t>
         </is>
       </c>
     </row>
@@ -3895,7 +3895,7 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>0.19s</t>
+          <t>0.21s</t>
         </is>
       </c>
     </row>
@@ -3932,7 +3932,7 @@
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>0.46s</t>
+          <t>0.44s</t>
         </is>
       </c>
     </row>
@@ -3969,7 +3969,7 @@
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>0.42s</t>
+          <t>0.18s</t>
         </is>
       </c>
     </row>
@@ -4006,7 +4006,7 @@
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>0.44s</t>
+          <t>0.20s</t>
         </is>
       </c>
     </row>
@@ -4043,7 +4043,7 @@
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.46s</t>
         </is>
       </c>
     </row>
@@ -4080,7 +4080,7 @@
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>0.15s</t>
+          <t>0.47s</t>
         </is>
       </c>
     </row>
@@ -4117,7 +4117,7 @@
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>0.31s</t>
+          <t>0.34s</t>
         </is>
       </c>
     </row>
@@ -4154,7 +4154,7 @@
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>0.30s</t>
+          <t>0.12s</t>
         </is>
       </c>
     </row>
@@ -4191,7 +4191,7 @@
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>0.19s</t>
+          <t>0.20s</t>
         </is>
       </c>
     </row>
@@ -4228,7 +4228,7 @@
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>0.50s</t>
+          <t>0.26s</t>
         </is>
       </c>
     </row>
@@ -4265,7 +4265,7 @@
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>0.10s</t>
+          <t>0.27s</t>
         </is>
       </c>
     </row>
@@ -4302,7 +4302,7 @@
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>0.13s</t>
+          <t>0.31s</t>
         </is>
       </c>
     </row>
@@ -4339,7 +4339,7 @@
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>0.25s</t>
+          <t>0.27s</t>
         </is>
       </c>
     </row>
@@ -4376,7 +4376,7 @@
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>0.37s</t>
+          <t>0.48s</t>
         </is>
       </c>
     </row>
@@ -4413,7 +4413,7 @@
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>0.32s</t>
+          <t>0.41s</t>
         </is>
       </c>
     </row>
@@ -4450,7 +4450,7 @@
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>0.31s</t>
+          <t>0.27s</t>
         </is>
       </c>
     </row>
@@ -4487,7 +4487,7 @@
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>0.18s</t>
+          <t>0.30s</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>0.43s</t>
+          <t>0.42s</t>
         </is>
       </c>
     </row>
@@ -4561,7 +4561,7 @@
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>0.13s</t>
+          <t>0.15s</t>
         </is>
       </c>
     </row>
@@ -4598,7 +4598,7 @@
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>0.16s</t>
+          <t>0.47s</t>
         </is>
       </c>
     </row>
@@ -4635,7 +4635,7 @@
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>0.10s</t>
+          <t>0.41s</t>
         </is>
       </c>
     </row>
@@ -4672,7 +4672,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.19s</t>
         </is>
       </c>
     </row>
@@ -4709,7 +4709,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>0.15s</t>
+          <t>0.12s</t>
         </is>
       </c>
     </row>
@@ -4746,7 +4746,7 @@
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>0.10s</t>
+          <t>0.47s</t>
         </is>
       </c>
     </row>
@@ -4783,7 +4783,7 @@
       </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
-          <t>0.27s</t>
+          <t>0.28s</t>
         </is>
       </c>
     </row>
@@ -4820,7 +4820,7 @@
       </c>
       <c r="G114" s="2" t="inlineStr">
         <is>
-          <t>0.43s</t>
+          <t>0.39s</t>
         </is>
       </c>
     </row>
@@ -4857,7 +4857,7 @@
       </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
-          <t>0.18s</t>
+          <t>0.42s</t>
         </is>
       </c>
     </row>
@@ -4894,7 +4894,7 @@
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>0.18s</t>
+          <t>0.14s</t>
         </is>
       </c>
     </row>
@@ -4931,7 +4931,7 @@
       </c>
       <c r="G117" s="2" t="inlineStr">
         <is>
-          <t>0.23s</t>
+          <t>0.11s</t>
         </is>
       </c>
     </row>
@@ -4968,7 +4968,7 @@
       </c>
       <c r="G118" s="2" t="inlineStr">
         <is>
-          <t>0.39s</t>
+          <t>0.13s</t>
         </is>
       </c>
     </row>
@@ -5005,7 +5005,7 @@
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
-          <t>0.42s</t>
+          <t>0.23s</t>
         </is>
       </c>
     </row>
@@ -5042,7 +5042,7 @@
       </c>
       <c r="G120" s="2" t="inlineStr">
         <is>
-          <t>0.20s</t>
+          <t>0.23s</t>
         </is>
       </c>
     </row>
@@ -5079,7 +5079,7 @@
       </c>
       <c r="G121" s="2" t="inlineStr">
         <is>
-          <t>0.26s</t>
+          <t>0.18s</t>
         </is>
       </c>
     </row>
@@ -5116,7 +5116,7 @@
       </c>
       <c r="G122" s="2" t="inlineStr">
         <is>
-          <t>0.33s</t>
+          <t>0.36s</t>
         </is>
       </c>
     </row>
@@ -5153,7 +5153,7 @@
       </c>
       <c r="G123" s="2" t="inlineStr">
         <is>
-          <t>0.26s</t>
+          <t>0.31s</t>
         </is>
       </c>
     </row>
@@ -5190,7 +5190,7 @@
       </c>
       <c r="G124" s="2" t="inlineStr">
         <is>
-          <t>0.16s</t>
+          <t>0.46s</t>
         </is>
       </c>
     </row>
@@ -5227,7 +5227,7 @@
       </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.26s</t>
         </is>
       </c>
     </row>
@@ -5264,7 +5264,7 @@
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
-          <t>0.48s</t>
+          <t>0.22s</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="G127" s="2" t="inlineStr">
         <is>
-          <t>0.42s</t>
+          <t>0.33s</t>
         </is>
       </c>
     </row>
@@ -5338,7 +5338,7 @@
       </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
-          <t>0.34s</t>
+          <t>0.45s</t>
         </is>
       </c>
     </row>
@@ -5375,7 +5375,7 @@
       </c>
       <c r="G129" s="2" t="inlineStr">
         <is>
-          <t>0.16s</t>
+          <t>0.17s</t>
         </is>
       </c>
     </row>
@@ -5412,7 +5412,7 @@
       </c>
       <c r="G130" s="2" t="inlineStr">
         <is>
-          <t>0.36s</t>
+          <t>0.44s</t>
         </is>
       </c>
     </row>
@@ -5449,7 +5449,7 @@
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>0.43s</t>
+          <t>0.41s</t>
         </is>
       </c>
     </row>
@@ -5486,7 +5486,7 @@
       </c>
       <c r="G132" s="2" t="inlineStr">
         <is>
-          <t>0.42s</t>
+          <t>0.30s</t>
         </is>
       </c>
     </row>
@@ -5523,7 +5523,7 @@
       </c>
       <c r="G133" s="2" t="inlineStr">
         <is>
-          <t>0.25s</t>
+          <t>0.24s</t>
         </is>
       </c>
     </row>
@@ -5597,7 +5597,7 @@
       </c>
       <c r="G135" s="2" t="inlineStr">
         <is>
-          <t>0.15s</t>
+          <t>0.12s</t>
         </is>
       </c>
     </row>
@@ -5634,7 +5634,7 @@
       </c>
       <c r="G136" s="2" t="inlineStr">
         <is>
-          <t>0.24s</t>
+          <t>0.38s</t>
         </is>
       </c>
     </row>
@@ -5671,7 +5671,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>0.36s</t>
+          <t>0.33s</t>
         </is>
       </c>
     </row>
@@ -5708,7 +5708,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>0.26s</t>
+          <t>0.13s</t>
         </is>
       </c>
     </row>
@@ -5745,7 +5745,7 @@
       </c>
       <c r="G139" s="2" t="inlineStr">
         <is>
-          <t>0.16s</t>
+          <t>0.30s</t>
         </is>
       </c>
     </row>
@@ -5782,7 +5782,7 @@
       </c>
       <c r="G140" s="2" t="inlineStr">
         <is>
-          <t>0.44s</t>
+          <t>0.46s</t>
         </is>
       </c>
     </row>
@@ -5819,7 +5819,7 @@
       </c>
       <c r="G141" s="2" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.17s</t>
         </is>
       </c>
     </row>
@@ -5856,7 +5856,7 @@
       </c>
       <c r="G142" s="2" t="inlineStr">
         <is>
-          <t>0.46s</t>
+          <t>0.17s</t>
         </is>
       </c>
     </row>
@@ -5893,7 +5893,7 @@
       </c>
       <c r="G143" s="2" t="inlineStr">
         <is>
-          <t>0.45s</t>
+          <t>0.17s</t>
         </is>
       </c>
     </row>
@@ -5930,7 +5930,7 @@
       </c>
       <c r="G144" s="2" t="inlineStr">
         <is>
-          <t>0.35s</t>
+          <t>0.49s</t>
         </is>
       </c>
     </row>
@@ -5967,7 +5967,7 @@
       </c>
       <c r="G145" s="2" t="inlineStr">
         <is>
-          <t>0.43s</t>
+          <t>0.24s</t>
         </is>
       </c>
     </row>
@@ -6004,7 +6004,7 @@
       </c>
       <c r="G146" s="2" t="inlineStr">
         <is>
-          <t>0.32s</t>
+          <t>0.48s</t>
         </is>
       </c>
     </row>
@@ -6041,7 +6041,7 @@
       </c>
       <c r="G147" s="2" t="inlineStr">
         <is>
-          <t>0.35s</t>
+          <t>0.14s</t>
         </is>
       </c>
     </row>
@@ -6078,7 +6078,7 @@
       </c>
       <c r="G148" s="2" t="inlineStr">
         <is>
-          <t>0.14s</t>
+          <t>0.22s</t>
         </is>
       </c>
     </row>
@@ -6115,7 +6115,7 @@
       </c>
       <c r="G149" s="2" t="inlineStr">
         <is>
-          <t>0.19s</t>
+          <t>0.20s</t>
         </is>
       </c>
     </row>
@@ -6152,7 +6152,7 @@
       </c>
       <c r="G150" s="2" t="inlineStr">
         <is>
-          <t>0.34s</t>
+          <t>0.15s</t>
         </is>
       </c>
     </row>
@@ -6189,7 +6189,7 @@
       </c>
       <c r="G151" s="2" t="inlineStr">
         <is>
-          <t>0.26s</t>
+          <t>0.25s</t>
         </is>
       </c>
     </row>
@@ -6226,7 +6226,7 @@
       </c>
       <c r="G152" s="2" t="inlineStr">
         <is>
-          <t>0.21s</t>
+          <t>0.30s</t>
         </is>
       </c>
     </row>
@@ -6263,7 +6263,7 @@
       </c>
       <c r="G153" s="2" t="inlineStr">
         <is>
-          <t>0.34s</t>
+          <t>0.45s</t>
         </is>
       </c>
     </row>
@@ -6300,7 +6300,7 @@
       </c>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>0.30s</t>
+          <t>0.33s</t>
         </is>
       </c>
     </row>
@@ -6337,7 +6337,7 @@
       </c>
       <c r="G155" s="2" t="inlineStr">
         <is>
-          <t>0.19s</t>
+          <t>0.47s</t>
         </is>
       </c>
     </row>
@@ -6374,7 +6374,7 @@
       </c>
       <c r="G156" s="2" t="inlineStr">
         <is>
-          <t>0.48s</t>
+          <t>0.11s</t>
         </is>
       </c>
     </row>
@@ -6411,7 +6411,7 @@
       </c>
       <c r="G157" s="2" t="inlineStr">
         <is>
-          <t>0.22s</t>
+          <t>0.34s</t>
         </is>
       </c>
     </row>
@@ -6448,7 +6448,7 @@
       </c>
       <c r="G158" s="2" t="inlineStr">
         <is>
-          <t>0.40s</t>
+          <t>0.15s</t>
         </is>
       </c>
     </row>
@@ -6485,7 +6485,7 @@
       </c>
       <c r="G159" s="2" t="inlineStr">
         <is>
-          <t>0.40s</t>
+          <t>0.36s</t>
         </is>
       </c>
     </row>
@@ -6522,7 +6522,7 @@
       </c>
       <c r="G160" s="2" t="inlineStr">
         <is>
-          <t>0.30s</t>
+          <t>0.10s</t>
         </is>
       </c>
     </row>
@@ -6559,7 +6559,7 @@
       </c>
       <c r="G161" s="2" t="inlineStr">
         <is>
-          <t>0.26s</t>
+          <t>0.21s</t>
         </is>
       </c>
     </row>
@@ -6596,7 +6596,7 @@
       </c>
       <c r="G162" s="2" t="inlineStr">
         <is>
-          <t>0.15s</t>
+          <t>0.17s</t>
         </is>
       </c>
     </row>
@@ -6633,7 +6633,7 @@
       </c>
       <c r="G163" s="2" t="inlineStr">
         <is>
-          <t>0.32s</t>
+          <t>0.16s</t>
         </is>
       </c>
     </row>
@@ -6670,7 +6670,7 @@
       </c>
       <c r="G164" s="2" t="inlineStr">
         <is>
-          <t>0.48s</t>
+          <t>0.34s</t>
         </is>
       </c>
     </row>
@@ -6707,7 +6707,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>0.27s</t>
+          <t>0.26s</t>
         </is>
       </c>
     </row>
@@ -6744,7 +6744,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>0.31s</t>
+          <t>0.44s</t>
         </is>
       </c>
     </row>
@@ -6781,7 +6781,7 @@
       </c>
       <c r="G167" s="2" t="inlineStr">
         <is>
-          <t>0.22s</t>
+          <t>0.34s</t>
         </is>
       </c>
     </row>
@@ -6818,7 +6818,7 @@
       </c>
       <c r="G168" s="2" t="inlineStr">
         <is>
-          <t>0.36s</t>
+          <t>0.11s</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="G169" s="2" t="inlineStr">
         <is>
-          <t>0.30s</t>
+          <t>0.12s</t>
         </is>
       </c>
     </row>
@@ -6892,7 +6892,7 @@
       </c>
       <c r="G170" s="2" t="inlineStr">
         <is>
-          <t>0.40s</t>
+          <t>0.45s</t>
         </is>
       </c>
     </row>
@@ -6929,7 +6929,7 @@
       </c>
       <c r="G171" s="2" t="inlineStr">
         <is>
-          <t>0.16s</t>
+          <t>0.27s</t>
         </is>
       </c>
     </row>
@@ -6966,7 +6966,7 @@
       </c>
       <c r="G172" s="2" t="inlineStr">
         <is>
-          <t>0.31s</t>
+          <t>0.16s</t>
         </is>
       </c>
     </row>
@@ -7003,7 +7003,7 @@
       </c>
       <c r="G173" s="2" t="inlineStr">
         <is>
-          <t>0.39s</t>
+          <t>0.19s</t>
         </is>
       </c>
     </row>
@@ -7040,7 +7040,7 @@
       </c>
       <c r="G174" s="2" t="inlineStr">
         <is>
-          <t>0.11s</t>
+          <t>0.35s</t>
         </is>
       </c>
     </row>
@@ -7077,7 +7077,7 @@
       </c>
       <c r="G175" s="2" t="inlineStr">
         <is>
-          <t>0.16s</t>
+          <t>0.30s</t>
         </is>
       </c>
     </row>
@@ -7114,7 +7114,7 @@
       </c>
       <c r="G176" s="2" t="inlineStr">
         <is>
-          <t>0.17s</t>
+          <t>0.14s</t>
         </is>
       </c>
     </row>
@@ -7151,7 +7151,7 @@
       </c>
       <c r="G177" s="2" t="inlineStr">
         <is>
-          <t>0.14s</t>
+          <t>0.25s</t>
         </is>
       </c>
     </row>
@@ -7188,7 +7188,7 @@
       </c>
       <c r="G178" s="2" t="inlineStr">
         <is>
-          <t>0.33s</t>
+          <t>0.31s</t>
         </is>
       </c>
     </row>
@@ -7225,7 +7225,7 @@
       </c>
       <c r="G179" s="2" t="inlineStr">
         <is>
-          <t>0.45s</t>
+          <t>0.27s</t>
         </is>
       </c>
     </row>
@@ -7262,7 +7262,7 @@
       </c>
       <c r="G180" s="2" t="inlineStr">
         <is>
-          <t>0.44s</t>
+          <t>0.45s</t>
         </is>
       </c>
     </row>
@@ -7299,7 +7299,7 @@
       </c>
       <c r="G181" s="2" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.28s</t>
         </is>
       </c>
     </row>
@@ -7336,7 +7336,7 @@
       </c>
       <c r="G182" s="2" t="inlineStr">
         <is>
-          <t>0.33s</t>
+          <t>0.26s</t>
         </is>
       </c>
     </row>
@@ -7373,7 +7373,7 @@
       </c>
       <c r="G183" s="2" t="inlineStr">
         <is>
-          <t>0.27s</t>
+          <t>0.21s</t>
         </is>
       </c>
     </row>
@@ -7410,7 +7410,7 @@
       </c>
       <c r="G184" s="2" t="inlineStr">
         <is>
-          <t>0.39s</t>
+          <t>0.26s</t>
         </is>
       </c>
     </row>
@@ -7447,7 +7447,7 @@
       </c>
       <c r="G185" s="2" t="inlineStr">
         <is>
-          <t>0.29s</t>
+          <t>0.28s</t>
         </is>
       </c>
     </row>
@@ -7484,7 +7484,7 @@
       </c>
       <c r="G186" s="2" t="inlineStr">
         <is>
-          <t>0.20s</t>
+          <t>0.24s</t>
         </is>
       </c>
     </row>
@@ -7521,7 +7521,7 @@
       </c>
       <c r="G187" s="2" t="inlineStr">
         <is>
-          <t>0.15s</t>
+          <t>0.14s</t>
         </is>
       </c>
     </row>
@@ -7558,7 +7558,7 @@
       </c>
       <c r="G188" s="2" t="inlineStr">
         <is>
-          <t>0.23s</t>
+          <t>0.26s</t>
         </is>
       </c>
     </row>
@@ -7595,7 +7595,7 @@
       </c>
       <c r="G189" s="2" t="inlineStr">
         <is>
-          <t>0.43s</t>
+          <t>0.46s</t>
         </is>
       </c>
     </row>
@@ -7632,7 +7632,7 @@
       </c>
       <c r="G190" s="2" t="inlineStr">
         <is>
-          <t>0.14s</t>
+          <t>0.26s</t>
         </is>
       </c>
     </row>
@@ -7669,7 +7669,7 @@
       </c>
       <c r="G191" s="2" t="inlineStr">
         <is>
-          <t>0.44s</t>
+          <t>0.46s</t>
         </is>
       </c>
     </row>
@@ -7706,7 +7706,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>0.32s</t>
+          <t>0.45s</t>
         </is>
       </c>
     </row>
@@ -7743,7 +7743,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>0.33s</t>
+          <t>0.17s</t>
         </is>
       </c>
     </row>
@@ -7780,7 +7780,7 @@
       </c>
       <c r="G194" s="2" t="inlineStr">
         <is>
-          <t>0.10s</t>
+          <t>0.36s</t>
         </is>
       </c>
     </row>
@@ -7817,7 +7817,7 @@
       </c>
       <c r="G195" s="2" t="inlineStr">
         <is>
-          <t>0.26s</t>
+          <t>0.33s</t>
         </is>
       </c>
     </row>
@@ -7854,7 +7854,7 @@
       </c>
       <c r="G196" s="2" t="inlineStr">
         <is>
-          <t>0.14s</t>
+          <t>0.21s</t>
         </is>
       </c>
     </row>
@@ -7891,7 +7891,7 @@
       </c>
       <c r="G197" s="2" t="inlineStr">
         <is>
-          <t>0.43s</t>
+          <t>0.46s</t>
         </is>
       </c>
     </row>
@@ -7928,7 +7928,7 @@
       </c>
       <c r="G198" s="2" t="inlineStr">
         <is>
-          <t>0.16s</t>
+          <t>0.21s</t>
         </is>
       </c>
     </row>
@@ -7965,7 +7965,7 @@
       </c>
       <c r="G199" s="2" t="inlineStr">
         <is>
-          <t>0.22s</t>
+          <t>0.14s</t>
         </is>
       </c>
     </row>
@@ -8002,7 +8002,7 @@
       </c>
       <c r="G200" s="2" t="inlineStr">
         <is>
-          <t>0.37s</t>
+          <t>0.27s</t>
         </is>
       </c>
     </row>
@@ -8039,7 +8039,7 @@
       </c>
       <c r="G201" s="2" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.20s</t>
         </is>
       </c>
     </row>
@@ -8076,7 +8076,7 @@
       </c>
       <c r="G202" s="2" t="inlineStr">
         <is>
-          <t>0.16s</t>
+          <t>0.43s</t>
         </is>
       </c>
     </row>
@@ -8113,7 +8113,7 @@
       </c>
       <c r="G203" s="2" t="inlineStr">
         <is>
-          <t>0.36s</t>
+          <t>0.21s</t>
         </is>
       </c>
     </row>
@@ -8150,7 +8150,7 @@
       </c>
       <c r="G204" s="2" t="inlineStr">
         <is>
-          <t>0.48s</t>
+          <t>0.45s</t>
         </is>
       </c>
     </row>
@@ -8187,7 +8187,7 @@
       </c>
       <c r="G205" s="2" t="inlineStr">
         <is>
-          <t>0.44s</t>
+          <t>0.48s</t>
         </is>
       </c>
     </row>
@@ -8224,7 +8224,7 @@
       </c>
       <c r="G206" s="2" t="inlineStr">
         <is>
-          <t>0.43s</t>
+          <t>0.34s</t>
         </is>
       </c>
     </row>
@@ -8261,7 +8261,7 @@
       </c>
       <c r="G207" s="2" t="inlineStr">
         <is>
-          <t>0.29s</t>
+          <t>0.11s</t>
         </is>
       </c>
     </row>
@@ -8298,7 +8298,7 @@
       </c>
       <c r="G208" s="2" t="inlineStr">
         <is>
-          <t>0.15s</t>
+          <t>0.21s</t>
         </is>
       </c>
     </row>
@@ -8335,7 +8335,7 @@
       </c>
       <c r="G209" s="2" t="inlineStr">
         <is>
-          <t>0.31s</t>
+          <t>0.32s</t>
         </is>
       </c>
     </row>
@@ -8372,7 +8372,7 @@
       </c>
       <c r="G210" s="2" t="inlineStr">
         <is>
-          <t>0.35s</t>
+          <t>0.36s</t>
         </is>
       </c>
     </row>
@@ -8409,7 +8409,7 @@
       </c>
       <c r="G211" s="2" t="inlineStr">
         <is>
-          <t>0.28s</t>
+          <t>0.23s</t>
         </is>
       </c>
     </row>
@@ -8446,7 +8446,7 @@
       </c>
       <c r="G212" s="2" t="inlineStr">
         <is>
-          <t>0.37s</t>
+          <t>0.43s</t>
         </is>
       </c>
     </row>
@@ -8483,7 +8483,7 @@
       </c>
       <c r="G213" s="2" t="inlineStr">
         <is>
-          <t>0.24s</t>
+          <t>0.36s</t>
         </is>
       </c>
     </row>
@@ -8520,7 +8520,7 @@
       </c>
       <c r="G214" s="2" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.18s</t>
         </is>
       </c>
     </row>
@@ -8557,7 +8557,7 @@
       </c>
       <c r="G215" s="2" t="inlineStr">
         <is>
-          <t>0.22s</t>
+          <t>0.44s</t>
         </is>
       </c>
     </row>
@@ -8594,7 +8594,7 @@
       </c>
       <c r="G216" s="2" t="inlineStr">
         <is>
-          <t>0.15s</t>
+          <t>0.14s</t>
         </is>
       </c>
     </row>
@@ -8631,7 +8631,7 @@
       </c>
       <c r="G217" s="2" t="inlineStr">
         <is>
-          <t>0.17s</t>
+          <t>0.37s</t>
         </is>
       </c>
     </row>
@@ -8668,7 +8668,7 @@
       </c>
       <c r="G218" s="2" t="inlineStr">
         <is>
-          <t>0.23s</t>
+          <t>0.15s</t>
         </is>
       </c>
     </row>
@@ -8705,7 +8705,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.11s</t>
         </is>
       </c>
     </row>
@@ -8742,7 +8742,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>0.32s</t>
+          <t>0.27s</t>
         </is>
       </c>
     </row>
@@ -8779,7 +8779,7 @@
       </c>
       <c r="G221" s="2" t="inlineStr">
         <is>
-          <t>0.30s</t>
+          <t>0.18s</t>
         </is>
       </c>
     </row>
@@ -8816,7 +8816,7 @@
       </c>
       <c r="G222" s="2" t="inlineStr">
         <is>
-          <t>0.22s</t>
+          <t>0.24s</t>
         </is>
       </c>
     </row>
@@ -8853,7 +8853,7 @@
       </c>
       <c r="G223" s="2" t="inlineStr">
         <is>
-          <t>0.20s</t>
+          <t>0.34s</t>
         </is>
       </c>
     </row>
@@ -8890,7 +8890,7 @@
       </c>
       <c r="G224" s="2" t="inlineStr">
         <is>
-          <t>0.26s</t>
+          <t>0.20s</t>
         </is>
       </c>
     </row>
@@ -8927,7 +8927,7 @@
       </c>
       <c r="G225" s="2" t="inlineStr">
         <is>
-          <t>0.50s</t>
+          <t>0.24s</t>
         </is>
       </c>
     </row>
@@ -8964,7 +8964,7 @@
       </c>
       <c r="G226" s="2" t="inlineStr">
         <is>
-          <t>0.37s</t>
+          <t>0.20s</t>
         </is>
       </c>
     </row>
@@ -9001,7 +9001,7 @@
       </c>
       <c r="G227" s="2" t="inlineStr">
         <is>
-          <t>0.25s</t>
+          <t>0.26s</t>
         </is>
       </c>
     </row>
@@ -9038,7 +9038,7 @@
       </c>
       <c r="G228" s="2" t="inlineStr">
         <is>
-          <t>0.48s</t>
+          <t>0.32s</t>
         </is>
       </c>
     </row>
@@ -9075,7 +9075,7 @@
       </c>
       <c r="G229" s="2" t="inlineStr">
         <is>
-          <t>0.35s</t>
+          <t>0.45s</t>
         </is>
       </c>
     </row>
@@ -9112,7 +9112,7 @@
       </c>
       <c r="G230" s="2" t="inlineStr">
         <is>
-          <t>0.25s</t>
+          <t>0.16s</t>
         </is>
       </c>
     </row>
@@ -9149,7 +9149,7 @@
       </c>
       <c r="G231" s="2" t="inlineStr">
         <is>
-          <t>0.15s</t>
+          <t>0.47s</t>
         </is>
       </c>
     </row>
@@ -9186,7 +9186,7 @@
       </c>
       <c r="G232" s="2" t="inlineStr">
         <is>
-          <t>0.36s</t>
+          <t>0.23s</t>
         </is>
       </c>
     </row>
@@ -9223,7 +9223,7 @@
       </c>
       <c r="G233" s="2" t="inlineStr">
         <is>
-          <t>0.31s</t>
+          <t>0.15s</t>
         </is>
       </c>
     </row>
@@ -9260,7 +9260,7 @@
       </c>
       <c r="G234" s="2" t="inlineStr">
         <is>
-          <t>0.35s</t>
+          <t>0.12s</t>
         </is>
       </c>
     </row>
@@ -9297,7 +9297,7 @@
       </c>
       <c r="G235" s="2" t="inlineStr">
         <is>
-          <t>0.15s</t>
+          <t>0.41s</t>
         </is>
       </c>
     </row>
@@ -9334,7 +9334,7 @@
       </c>
       <c r="G236" s="2" t="inlineStr">
         <is>
-          <t>0.20s</t>
+          <t>0.31s</t>
         </is>
       </c>
     </row>
@@ -9408,7 +9408,7 @@
       </c>
       <c r="G238" s="2" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.31s</t>
         </is>
       </c>
     </row>
@@ -9445,7 +9445,7 @@
       </c>
       <c r="G239" s="2" t="inlineStr">
         <is>
-          <t>0.50s</t>
+          <t>0.31s</t>
         </is>
       </c>
     </row>
@@ -9482,7 +9482,7 @@
       </c>
       <c r="G240" s="2" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.41s</t>
         </is>
       </c>
     </row>
@@ -9519,7 +9519,7 @@
       </c>
       <c r="G241" s="2" t="inlineStr">
         <is>
-          <t>0.30s</t>
+          <t>0.50s</t>
         </is>
       </c>
     </row>
@@ -9556,7 +9556,7 @@
       </c>
       <c r="G242" s="2" t="inlineStr">
         <is>
-          <t>0.25s</t>
+          <t>0.19s</t>
         </is>
       </c>
     </row>
@@ -9593,7 +9593,7 @@
       </c>
       <c r="G243" s="2" t="inlineStr">
         <is>
-          <t>0.24s</t>
+          <t>0.10s</t>
         </is>
       </c>
     </row>
@@ -9630,7 +9630,7 @@
       </c>
       <c r="G244" s="2" t="inlineStr">
         <is>
-          <t>0.13s</t>
+          <t>0.48s</t>
         </is>
       </c>
     </row>
@@ -9667,7 +9667,7 @@
       </c>
       <c r="G245" s="2" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.46s</t>
         </is>
       </c>
     </row>
@@ -9704,7 +9704,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>0.18s</t>
+          <t>0.15s</t>
         </is>
       </c>
     </row>
@@ -9741,7 +9741,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>0.47s</t>
+          <t>0.13s</t>
         </is>
       </c>
     </row>
@@ -9815,7 +9815,7 @@
       </c>
       <c r="G249" s="2" t="inlineStr">
         <is>
-          <t>0.21s</t>
+          <t>0.24s</t>
         </is>
       </c>
     </row>
@@ -9852,7 +9852,7 @@
       </c>
       <c r="G250" s="2" t="inlineStr">
         <is>
-          <t>0.28s</t>
+          <t>0.24s</t>
         </is>
       </c>
     </row>
@@ -9889,7 +9889,7 @@
       </c>
       <c r="G251" s="2" t="inlineStr">
         <is>
-          <t>0.14s</t>
+          <t>0.36s</t>
         </is>
       </c>
     </row>
@@ -9926,7 +9926,7 @@
       </c>
       <c r="G252" s="2" t="inlineStr">
         <is>
-          <t>0.20s</t>
+          <t>0.28s</t>
         </is>
       </c>
     </row>
@@ -9963,7 +9963,7 @@
       </c>
       <c r="G253" s="2" t="inlineStr">
         <is>
-          <t>0.49s</t>
+          <t>0.25s</t>
         </is>
       </c>
     </row>
@@ -10000,7 +10000,7 @@
       </c>
       <c r="G254" s="2" t="inlineStr">
         <is>
-          <t>0.39s</t>
+          <t>0.47s</t>
         </is>
       </c>
     </row>
@@ -10037,7 +10037,7 @@
       </c>
       <c r="G255" s="2" t="inlineStr">
         <is>
-          <t>0.36s</t>
+          <t>0.19s</t>
         </is>
       </c>
     </row>
@@ -10074,7 +10074,7 @@
       </c>
       <c r="G256" s="2" t="inlineStr">
         <is>
-          <t>0.31s</t>
+          <t>0.41s</t>
         </is>
       </c>
     </row>
@@ -10111,7 +10111,7 @@
       </c>
       <c r="G257" s="2" t="inlineStr">
         <is>
-          <t>0.27s</t>
+          <t>0.18s</t>
         </is>
       </c>
     </row>
@@ -10148,7 +10148,7 @@
       </c>
       <c r="G258" s="2" t="inlineStr">
         <is>
-          <t>0.48s</t>
+          <t>0.49s</t>
         </is>
       </c>
     </row>
@@ -10185,7 +10185,7 @@
       </c>
       <c r="G259" s="2" t="inlineStr">
         <is>
-          <t>0.36s</t>
+          <t>0.29s</t>
         </is>
       </c>
     </row>
@@ -10222,7 +10222,7 @@
       </c>
       <c r="G260" s="2" t="inlineStr">
         <is>
-          <t>0.11s</t>
+          <t>0.18s</t>
         </is>
       </c>
     </row>
@@ -10259,7 +10259,7 @@
       </c>
       <c r="G261" s="2" t="inlineStr">
         <is>
-          <t>0.26s</t>
+          <t>0.27s</t>
         </is>
       </c>
     </row>
@@ -10296,7 +10296,7 @@
       </c>
       <c r="G262" s="2" t="inlineStr">
         <is>
-          <t>0.42s</t>
+          <t>0.32s</t>
         </is>
       </c>
     </row>
@@ -10333,7 +10333,7 @@
       </c>
       <c r="G263" s="2" t="inlineStr">
         <is>
-          <t>0.21s</t>
+          <t>0.42s</t>
         </is>
       </c>
     </row>
@@ -10370,7 +10370,7 @@
       </c>
       <c r="G264" s="2" t="inlineStr">
         <is>
-          <t>0.30s</t>
+          <t>0.25s</t>
         </is>
       </c>
     </row>
@@ -10407,7 +10407,7 @@
       </c>
       <c r="G265" s="2" t="inlineStr">
         <is>
-          <t>0.27s</t>
+          <t>0.31s</t>
         </is>
       </c>
     </row>
@@ -10444,7 +10444,7 @@
       </c>
       <c r="G266" s="2" t="inlineStr">
         <is>
-          <t>0.24s</t>
+          <t>0.12s</t>
         </is>
       </c>
     </row>
@@ -10481,7 +10481,7 @@
       </c>
       <c r="G267" s="2" t="inlineStr">
         <is>
-          <t>0.14s</t>
+          <t>0.43s</t>
         </is>
       </c>
     </row>
@@ -10518,7 +10518,7 @@
       </c>
       <c r="G268" s="2" t="inlineStr">
         <is>
-          <t>0.38s</t>
+          <t>0.10s</t>
         </is>
       </c>
     </row>
@@ -10555,7 +10555,7 @@
       </c>
       <c r="G269" s="2" t="inlineStr">
         <is>
-          <t>0.15s</t>
+          <t>0.14s</t>
         </is>
       </c>
     </row>
@@ -10592,7 +10592,7 @@
       </c>
       <c r="G270" s="2" t="inlineStr">
         <is>
-          <t>0.38s</t>
+          <t>0.47s</t>
         </is>
       </c>
     </row>
@@ -10629,7 +10629,7 @@
       </c>
       <c r="G271" s="2" t="inlineStr">
         <is>
-          <t>0.39s</t>
+          <t>0.11s</t>
         </is>
       </c>
     </row>
@@ -10666,7 +10666,7 @@
       </c>
       <c r="G272" s="2" t="inlineStr">
         <is>
-          <t>0.47s</t>
+          <t>0.38s</t>
         </is>
       </c>
     </row>
@@ -10703,7 +10703,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>0.26s</t>
+          <t>0.38s</t>
         </is>
       </c>
     </row>
@@ -10740,7 +10740,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>0.27s</t>
+          <t>0.31s</t>
         </is>
       </c>
     </row>
@@ -10777,7 +10777,7 @@
       </c>
       <c r="G275" s="2" t="inlineStr">
         <is>
-          <t>0.22s</t>
+          <t>0.28s</t>
         </is>
       </c>
     </row>
@@ -10814,7 +10814,7 @@
       </c>
       <c r="G276" s="2" t="inlineStr">
         <is>
-          <t>0.40s</t>
+          <t>0.34s</t>
         </is>
       </c>
     </row>
@@ -10851,7 +10851,7 @@
       </c>
       <c r="G277" s="2" t="inlineStr">
         <is>
-          <t>0.38s</t>
+          <t>0.30s</t>
         </is>
       </c>
     </row>
@@ -10888,7 +10888,7 @@
       </c>
       <c r="G278" s="2" t="inlineStr">
         <is>
-          <t>0.35s</t>
+          <t>0.18s</t>
         </is>
       </c>
     </row>
@@ -10925,7 +10925,7 @@
       </c>
       <c r="G279" s="2" t="inlineStr">
         <is>
-          <t>0.33s</t>
+          <t>0.43s</t>
         </is>
       </c>
     </row>
@@ -10962,7 +10962,7 @@
       </c>
       <c r="G280" s="2" t="inlineStr">
         <is>
-          <t>0.36s</t>
+          <t>0.10s</t>
         </is>
       </c>
     </row>
@@ -10999,7 +10999,7 @@
       </c>
       <c r="G281" s="2" t="inlineStr">
         <is>
-          <t>0.42s</t>
+          <t>0.47s</t>
         </is>
       </c>
     </row>
@@ -11036,7 +11036,7 @@
       </c>
       <c r="G282" s="2" t="inlineStr">
         <is>
-          <t>0.33s</t>
+          <t>0.13s</t>
         </is>
       </c>
     </row>
@@ -11073,7 +11073,7 @@
       </c>
       <c r="G283" s="2" t="inlineStr">
         <is>
-          <t>0.16s</t>
+          <t>0.42s</t>
         </is>
       </c>
     </row>
@@ -11110,7 +11110,7 @@
       </c>
       <c r="G284" s="2" t="inlineStr">
         <is>
-          <t>0.15s</t>
+          <t>0.28s</t>
         </is>
       </c>
     </row>
@@ -11147,7 +11147,7 @@
       </c>
       <c r="G285" s="2" t="inlineStr">
         <is>
-          <t>0.23s</t>
+          <t>0.48s</t>
         </is>
       </c>
     </row>
@@ -11184,7 +11184,7 @@
       </c>
       <c r="G286" s="2" t="inlineStr">
         <is>
-          <t>0.46s</t>
+          <t>0.24s</t>
         </is>
       </c>
     </row>
@@ -11221,7 +11221,7 @@
       </c>
       <c r="G287" s="2" t="inlineStr">
         <is>
-          <t>0.31s</t>
+          <t>0.28s</t>
         </is>
       </c>
     </row>
@@ -11258,7 +11258,7 @@
       </c>
       <c r="G288" s="2" t="inlineStr">
         <is>
-          <t>0.33s</t>
+          <t>0.44s</t>
         </is>
       </c>
     </row>
@@ -11295,7 +11295,7 @@
       </c>
       <c r="G289" s="2" t="inlineStr">
         <is>
-          <t>0.13s</t>
+          <t>0.47s</t>
         </is>
       </c>
     </row>
@@ -11332,7 +11332,7 @@
       </c>
       <c r="G290" s="2" t="inlineStr">
         <is>
-          <t>0.22s</t>
+          <t>0.25s</t>
         </is>
       </c>
     </row>
@@ -11369,7 +11369,7 @@
       </c>
       <c r="G291" s="2" t="inlineStr">
         <is>
-          <t>0.29s</t>
+          <t>0.23s</t>
         </is>
       </c>
     </row>
@@ -11406,7 +11406,7 @@
       </c>
       <c r="G292" s="2" t="inlineStr">
         <is>
-          <t>0.24s</t>
+          <t>0.28s</t>
         </is>
       </c>
     </row>
@@ -11443,7 +11443,7 @@
       </c>
       <c r="G293" s="2" t="inlineStr">
         <is>
-          <t>0.17s</t>
+          <t>0.19s</t>
         </is>
       </c>
     </row>
@@ -11480,7 +11480,7 @@
       </c>
       <c r="G294" s="2" t="inlineStr">
         <is>
-          <t>0.28s</t>
+          <t>0.41s</t>
         </is>
       </c>
     </row>
@@ -11517,7 +11517,7 @@
       </c>
       <c r="G295" s="2" t="inlineStr">
         <is>
-          <t>0.38s</t>
+          <t>0.47s</t>
         </is>
       </c>
     </row>
@@ -11554,7 +11554,7 @@
       </c>
       <c r="G296" s="2" t="inlineStr">
         <is>
-          <t>0.18s</t>
+          <t>0.50s</t>
         </is>
       </c>
     </row>
@@ -11591,7 +11591,7 @@
       </c>
       <c r="G297" s="2" t="inlineStr">
         <is>
-          <t>0.15s</t>
+          <t>0.22s</t>
         </is>
       </c>
     </row>
@@ -11628,7 +11628,7 @@
       </c>
       <c r="G298" s="2" t="inlineStr">
         <is>
-          <t>0.44s</t>
+          <t>0.24s</t>
         </is>
       </c>
     </row>
@@ -11665,7 +11665,7 @@
       </c>
       <c r="G299" s="2" t="inlineStr">
         <is>
-          <t>0.23s</t>
+          <t>0.38s</t>
         </is>
       </c>
     </row>
@@ -11702,7 +11702,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>0.40s</t>
+          <t>0.29s</t>
         </is>
       </c>
     </row>
@@ -11739,7 +11739,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>0.25s</t>
+          <t>0.32s</t>
         </is>
       </c>
     </row>
@@ -11776,7 +11776,7 @@
       </c>
       <c r="G302" s="2" t="inlineStr">
         <is>
-          <t>0.29s</t>
+          <t>0.34s</t>
         </is>
       </c>
     </row>
@@ -11813,7 +11813,7 @@
       </c>
       <c r="G303" s="2" t="inlineStr">
         <is>
-          <t>0.42s</t>
+          <t>0.29s</t>
         </is>
       </c>
     </row>
@@ -11850,7 +11850,7 @@
       </c>
       <c r="G304" s="2" t="inlineStr">
         <is>
-          <t>0.22s</t>
+          <t>0.10s</t>
         </is>
       </c>
     </row>
@@ -11887,7 +11887,7 @@
       </c>
       <c r="G305" s="2" t="inlineStr">
         <is>
-          <t>0.37s</t>
+          <t>0.24s</t>
         </is>
       </c>
     </row>
@@ -11924,7 +11924,7 @@
       </c>
       <c r="G306" s="2" t="inlineStr">
         <is>
-          <t>0.32s</t>
+          <t>0.37s</t>
         </is>
       </c>
     </row>
@@ -11961,7 +11961,7 @@
       </c>
       <c r="G307" s="2" t="inlineStr">
         <is>
-          <t>0.34s</t>
+          <t>0.43s</t>
         </is>
       </c>
     </row>
@@ -11998,7 +11998,7 @@
       </c>
       <c r="G308" s="2" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.36s</t>
         </is>
       </c>
     </row>
@@ -12035,7 +12035,7 @@
       </c>
       <c r="G309" s="2" t="inlineStr">
         <is>
-          <t>0.29s</t>
+          <t>0.46s</t>
         </is>
       </c>
     </row>
@@ -12072,7 +12072,7 @@
       </c>
       <c r="G310" s="2" t="inlineStr">
         <is>
-          <t>0.24s</t>
+          <t>0.22s</t>
         </is>
       </c>
     </row>
@@ -12109,7 +12109,7 @@
       </c>
       <c r="G311" s="2" t="inlineStr">
         <is>
-          <t>0.17s</t>
+          <t>0.38s</t>
         </is>
       </c>
     </row>
@@ -12146,7 +12146,7 @@
       </c>
       <c r="G312" s="2" t="inlineStr">
         <is>
-          <t>0.14s</t>
+          <t>0.17s</t>
         </is>
       </c>
     </row>
@@ -12183,7 +12183,7 @@
       </c>
       <c r="G313" s="2" t="inlineStr">
         <is>
-          <t>0.16s</t>
+          <t>0.36s</t>
         </is>
       </c>
     </row>
@@ -12220,7 +12220,7 @@
       </c>
       <c r="G314" s="2" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.33s</t>
         </is>
       </c>
     </row>
@@ -12257,7 +12257,7 @@
       </c>
       <c r="G315" s="2" t="inlineStr">
         <is>
-          <t>0.25s</t>
+          <t>0.45s</t>
         </is>
       </c>
     </row>
@@ -12294,7 +12294,7 @@
       </c>
       <c r="G316" s="2" t="inlineStr">
         <is>
-          <t>0.45s</t>
+          <t>0.40s</t>
         </is>
       </c>
     </row>
@@ -12331,7 +12331,7 @@
       </c>
       <c r="G317" s="2" t="inlineStr">
         <is>
-          <t>0.31s</t>
+          <t>0.45s</t>
         </is>
       </c>
     </row>
@@ -12368,7 +12368,7 @@
       </c>
       <c r="G318" s="2" t="inlineStr">
         <is>
-          <t>0.27s</t>
+          <t>0.26s</t>
         </is>
       </c>
     </row>
@@ -12405,7 +12405,7 @@
       </c>
       <c r="G319" s="2" t="inlineStr">
         <is>
-          <t>0.19s</t>
+          <t>0.26s</t>
         </is>
       </c>
     </row>
@@ -12479,7 +12479,7 @@
       </c>
       <c r="G321" s="2" t="inlineStr">
         <is>
-          <t>0.33s</t>
+          <t>0.45s</t>
         </is>
       </c>
     </row>
@@ -12516,7 +12516,7 @@
       </c>
       <c r="G322" s="2" t="inlineStr">
         <is>
-          <t>0.50s</t>
+          <t>0.43s</t>
         </is>
       </c>
     </row>
@@ -12553,7 +12553,7 @@
       </c>
       <c r="G323" s="2" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.30s</t>
         </is>
       </c>
     </row>
@@ -12590,7 +12590,7 @@
       </c>
       <c r="G324" s="2" t="inlineStr">
         <is>
-          <t>0.46s</t>
+          <t>0.28s</t>
         </is>
       </c>
     </row>
@@ -12627,7 +12627,7 @@
       </c>
       <c r="G325" s="2" t="inlineStr">
         <is>
-          <t>0.23s</t>
+          <t>0.12s</t>
         </is>
       </c>
     </row>
@@ -12664,7 +12664,7 @@
       </c>
       <c r="G326" s="2" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.24s</t>
         </is>
       </c>
     </row>
@@ -12701,7 +12701,7 @@
       </c>
       <c r="G327" s="2" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.17s</t>
         </is>
       </c>
     </row>
@@ -12738,7 +12738,7 @@
       </c>
       <c r="G328" s="2" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.20s</t>
         </is>
       </c>
     </row>
@@ -12775,7 +12775,7 @@
       </c>
       <c r="G329" s="2" t="inlineStr">
         <is>
-          <t>0.19s</t>
+          <t>0.43s</t>
         </is>
       </c>
     </row>
@@ -12812,7 +12812,7 @@
       </c>
       <c r="G330" s="2" t="inlineStr">
         <is>
-          <t>0.33s</t>
+          <t>0.25s</t>
         </is>
       </c>
     </row>
@@ -12849,7 +12849,7 @@
       </c>
       <c r="G331" s="2" t="inlineStr">
         <is>
-          <t>0.40s</t>
+          <t>0.32s</t>
         </is>
       </c>
     </row>
@@ -12886,7 +12886,7 @@
       </c>
       <c r="G332" s="2" t="inlineStr">
         <is>
-          <t>0.13s</t>
+          <t>0.26s</t>
         </is>
       </c>
     </row>
@@ -12923,7 +12923,7 @@
       </c>
       <c r="G333" s="2" t="inlineStr">
         <is>
-          <t>0.34s</t>
+          <t>0.23s</t>
         </is>
       </c>
     </row>
@@ -12960,7 +12960,7 @@
       </c>
       <c r="G334" s="2" t="inlineStr">
         <is>
-          <t>0.39s</t>
+          <t>0.50s</t>
         </is>
       </c>
     </row>
@@ -12997,7 +12997,7 @@
       </c>
       <c r="G335" s="2" t="inlineStr">
         <is>
-          <t>0.39s</t>
+          <t>0.49s</t>
         </is>
       </c>
     </row>
@@ -13034,7 +13034,7 @@
       </c>
       <c r="G336" s="2" t="inlineStr">
         <is>
-          <t>0.47s</t>
+          <t>0.38s</t>
         </is>
       </c>
     </row>
@@ -13071,7 +13071,7 @@
       </c>
       <c r="G337" s="2" t="inlineStr">
         <is>
-          <t>0.46s</t>
+          <t>0.18s</t>
         </is>
       </c>
     </row>
@@ -13108,7 +13108,7 @@
       </c>
       <c r="G338" s="2" t="inlineStr">
         <is>
-          <t>0.21s</t>
+          <t>0.44s</t>
         </is>
       </c>
     </row>
@@ -13145,7 +13145,7 @@
       </c>
       <c r="G339" s="2" t="inlineStr">
         <is>
-          <t>0.17s</t>
+          <t>0.31s</t>
         </is>
       </c>
     </row>
@@ -13182,7 +13182,7 @@
       </c>
       <c r="G340" s="2" t="inlineStr">
         <is>
-          <t>0.14s</t>
+          <t>0.26s</t>
         </is>
       </c>
     </row>
@@ -13219,7 +13219,7 @@
       </c>
       <c r="G341" s="2" t="inlineStr">
         <is>
-          <t>0.44s</t>
+          <t>0.18s</t>
         </is>
       </c>
     </row>
@@ -13256,7 +13256,7 @@
       </c>
       <c r="G342" s="2" t="inlineStr">
         <is>
-          <t>0.20s</t>
+          <t>0.48s</t>
         </is>
       </c>
     </row>
@@ -13293,7 +13293,7 @@
       </c>
       <c r="G343" s="2" t="inlineStr">
         <is>
-          <t>0.40s</t>
+          <t>0.22s</t>
         </is>
       </c>
     </row>
@@ -13330,7 +13330,7 @@
       </c>
       <c r="G344" s="2" t="inlineStr">
         <is>
-          <t>0.22s</t>
+          <t>0.40s</t>
         </is>
       </c>
     </row>
@@ -13367,7 +13367,7 @@
       </c>
       <c r="G345" s="2" t="inlineStr">
         <is>
-          <t>0.27s</t>
+          <t>0.16s</t>
         </is>
       </c>
     </row>
@@ -13404,7 +13404,7 @@
       </c>
       <c r="G346" s="2" t="inlineStr">
         <is>
-          <t>0.37s</t>
+          <t>0.35s</t>
         </is>
       </c>
     </row>
@@ -13441,7 +13441,7 @@
       </c>
       <c r="G347" s="2" t="inlineStr">
         <is>
-          <t>0.43s</t>
+          <t>0.44s</t>
         </is>
       </c>
     </row>
@@ -13478,7 +13478,7 @@
       </c>
       <c r="G348" s="2" t="inlineStr">
         <is>
-          <t>0.16s</t>
+          <t>0.47s</t>
         </is>
       </c>
     </row>
@@ -13515,7 +13515,7 @@
       </c>
       <c r="G349" s="2" t="inlineStr">
         <is>
-          <t>0.11s</t>
+          <t>0.22s</t>
         </is>
       </c>
     </row>
@@ -13552,7 +13552,7 @@
       </c>
       <c r="G350" s="2" t="inlineStr">
         <is>
-          <t>0.42s</t>
+          <t>0.33s</t>
         </is>
       </c>
     </row>
@@ -13589,7 +13589,7 @@
       </c>
       <c r="G351" s="2" t="inlineStr">
         <is>
-          <t>0.50s</t>
+          <t>0.44s</t>
         </is>
       </c>
     </row>
@@ -14324,7 +14324,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>103.90</t>
+          <t>104.26</t>
         </is>
       </c>
     </row>

</xml_diff>